<commit_message>
Sprint 1 Final Hours
</commit_message>
<xml_diff>
--- a/docs/AetherFlow_Sprint1_Final_Hours.xlsx
+++ b/docs/AetherFlow_Sprint1_Final_Hours.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\Documents\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FACF7176-A466-4FA1-AF5B-ED9621A2E98F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0705FD99-1ECE-4690-874A-D92E6FDE8F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="1" r:id="rId1"/>
@@ -53,9 +53,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="101">
-  <si>
-    <t>Airline Reservation System</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="101">
+  <si>
+    <t>Aether Flow</t>
   </si>
   <si>
     <t>What is this?</t>
@@ -6653,7 +6653,9 @@
       <c r="K13" s="28"/>
       <c r="L13" s="28"/>
       <c r="M13" s="30"/>
-      <c r="N13" s="28"/>
+      <c r="N13" s="28">
+        <v>2</v>
+      </c>
       <c r="O13" s="28"/>
       <c r="P13" s="28"/>
       <c r="Q13" s="28"/>
@@ -7248,23 +7250,23 @@
       </c>
       <c r="N24" s="9">
         <f>IF(SUM(N11:N23)&gt;0,E24-SUM(F11:N23),NA())</f>
-        <v>-25</v>
+        <v>-27</v>
       </c>
       <c r="O24" s="9">
         <f>IF(SUM(O11:O23)&gt;0,E24-SUM(F11:O23),NA())</f>
-        <v>-31</v>
+        <v>-33</v>
       </c>
       <c r="P24" s="9">
         <f>IF(SUM(P11:P23)&gt;0,E24-SUM(F11:P23),NA())</f>
-        <v>-39</v>
+        <v>-41</v>
       </c>
       <c r="Q24" s="9">
         <f>IF(SUM(Q11:Q23)&gt;0,E24-SUM(F11:Q23),NA())</f>
-        <v>-45</v>
+        <v>-47</v>
       </c>
       <c r="R24" s="9">
         <f>IF(SUM(R11:R23)&gt;0,E24-SUM(F11:R23),NA())</f>
-        <v>-55</v>
+        <v>-57</v>
       </c>
       <c r="S24" s="9" t="e">
         <f>IF(SUM(S11:S23)&gt;0,E24-SUM(F11:S23),NA())</f>
@@ -7699,7 +7701,9 @@
         <v>15</v>
       </c>
       <c r="D4" s="49"/>
-      <c r="E4" s="89"/>
+      <c r="E4" s="89" t="s">
+        <v>16</v>
+      </c>
       <c r="F4" s="90"/>
       <c r="G4" s="90"/>
       <c r="H4" s="90"/>

</xml_diff>